<commit_message>
Matching columns now not normalized
</commit_message>
<xml_diff>
--- a/samples/sample_1/SAFE_IC_INVENTORY_20251201.XLSX
+++ b/samples/sample_1/SAFE_IC_INVENTORY_20251201.XLSX
@@ -1,139 +1,154 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Sheet2" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Sheet3" state="visible" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
   <si>
-    <t>ITEM</t>
+    <t xml:space="preserve">ITEM</t>
   </si>
   <si>
-    <t>ITMDESC</t>
+    <t xml:space="preserve">ITMDESC</t>
   </si>
   <si>
-    <t>PLINID</t>
+    <t xml:space="preserve">PLINID</t>
   </si>
   <si>
-    <t>ITMCLSS</t>
+    <t xml:space="preserve">ITMCLSS</t>
   </si>
   <si>
-    <t>UPCCODE</t>
+    <t xml:space="preserve">UPCCODE</t>
   </si>
   <si>
-    <t>EDITION</t>
+    <t xml:space="preserve">EDITION</t>
   </si>
   <si>
-    <t>CURRDATE</t>
+    <t xml:space="preserve">CURRDATE</t>
   </si>
   <si>
-    <t>item 1</t>
+    <t xml:space="preserve">ITEM 1</t>
   </si>
   <si>
-    <t>chart</t>
+    <t xml:space="preserve">chart</t>
   </si>
   <si>
-    <t>abcd 1</t>
+    <t xml:space="preserve">abcd 1</t>
   </si>
   <si>
-    <t>ABC</t>
+    <t xml:space="preserve">ABC</t>
   </si>
   <si>
-    <t>1101</t>
+    <t xml:space="preserve">1101</t>
   </si>
   <si>
-    <t>2026</t>
+    <t xml:space="preserve">2026</t>
   </si>
   <si>
-    <t>01/01/2026</t>
+    <t xml:space="preserve">01/01/2026</t>
   </si>
   <si>
-    <t>item 2</t>
+    <t xml:space="preserve">ITEM 2</t>
   </si>
   <si>
-    <t>book</t>
+    <t xml:space="preserve">book</t>
   </si>
   <si>
-    <t>abcd 2</t>
+    <t xml:space="preserve">abcd 2</t>
   </si>
   <si>
-    <t>1102</t>
+    <t xml:space="preserve">1102</t>
   </si>
   <si>
-    <t>2025 (3)</t>
+    <t xml:space="preserve">2025 (3)</t>
   </si>
   <si>
-    <t>01/03/2025</t>
+    <t xml:space="preserve">01/03/2025</t>
   </si>
   <si>
-    <t>item 3</t>
+    <t xml:space="preserve">ITEM 3</t>
   </si>
   <si>
-    <t>software</t>
+    <t xml:space="preserve">software</t>
   </si>
   <si>
-    <t>abcd 3</t>
+    <t xml:space="preserve">abcd 3</t>
   </si>
   <si>
-    <t>1103</t>
+    <t xml:space="preserve">1103</t>
   </si>
   <si>
-    <t>1.2.0</t>
+    <t xml:space="preserve">1.2.0</t>
   </si>
   <si>
-    <t>item 4</t>
+    <t xml:space="preserve">ITEM 4</t>
   </si>
   <si>
-    <t>compass</t>
+    <t xml:space="preserve">compass</t>
   </si>
   <si>
-    <t>abcd 4</t>
+    <t xml:space="preserve">abcd 4</t>
   </si>
   <si>
-    <t>1104</t>
+    <t xml:space="preserve">1104</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <charset val="1"/>
     </font>
     <font>
-      <charset val="1"/>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -145,7 +160,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -153,34 +168,57 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -360,19 +398,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="18.71" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.71" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12" style="1" customWidth="1"/>
-    <col min="6" max="7" width="10.71" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="10.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -395,7 +436,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -418,7 +459,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -441,7 +482,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -462,7 +503,7 @@
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
@@ -480,2704 +521,2725 @@
       </c>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G6" s="3"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G7" s="3"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G8" s="3"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G9" s="3"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G10" s="3"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G11" s="3"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G12" s="3"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G13" s="3"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G17" s="3"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G18" s="3"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G20" s="3"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G21" s="3"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G22" s="3"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G24" s="3"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G26" s="3"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G27" s="3"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G31" s="3"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G32" s="3"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G33" s="3"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G34" s="3"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G35" s="3"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G36" s="3"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G37" s="3"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G38" s="3"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G39" s="3"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G42" s="3"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G43" s="3"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G45" s="3"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G46" s="3"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G48" s="3"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G49" s="3"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G52" s="3"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G55" s="3"/>
     </row>
-    <row r="57" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G57" s="3"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G58" s="3"/>
     </row>
-    <row r="59" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G59" s="3"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G60" s="3"/>
     </row>
-    <row r="61" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G61" s="3"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G62" s="3"/>
     </row>
-    <row r="63" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G63" s="3"/>
     </row>
-    <row r="65" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G65" s="3"/>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G67" s="3"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G68" s="3"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G70" s="3"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G72" s="3"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G73" s="3"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G74" s="3"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G76" s="3"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G77" s="3"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G78" s="3"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G79" s="3"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G80" s="3"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G83" s="3"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G87" s="3"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G90" s="3"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G91" s="3"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G92" s="3"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G94" s="3"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G95" s="3"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G96" s="3"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G98" s="3"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G99" s="3"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G100" s="3"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G101" s="3"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G102" s="3"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G103" s="3"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G104" s="3"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G105" s="3"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G106" s="3"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G107" s="3"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G109" s="3"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G112" s="3"/>
     </row>
-    <row r="115" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G115" s="3"/>
     </row>
-    <row r="116" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G116" s="3"/>
     </row>
-    <row r="117" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G117" s="3"/>
     </row>
-    <row r="118" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G118" s="3"/>
     </row>
-    <row r="119" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G119" s="3"/>
     </row>
-    <row r="120" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G120" s="3"/>
     </row>
-    <row r="121" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G121" s="3"/>
     </row>
-    <row r="122" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G122" s="3"/>
     </row>
-    <row r="123" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G123" s="3"/>
     </row>
-    <row r="124" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G124" s="3"/>
     </row>
-    <row r="125" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G125" s="3"/>
     </row>
-    <row r="126" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G126" s="3"/>
     </row>
-    <row r="127" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G127" s="3"/>
     </row>
-    <row r="128" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G128" s="3"/>
     </row>
-    <row r="129" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G129" s="3"/>
     </row>
-    <row r="130" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G130" s="3"/>
     </row>
-    <row r="132" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G132" s="3"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G133" s="3"/>
     </row>
-    <row r="134" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G134" s="3"/>
     </row>
-    <row r="135" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G135" s="3"/>
     </row>
-    <row r="136" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G136" s="3"/>
     </row>
-    <row r="137" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G137" s="3"/>
     </row>
-    <row r="140" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G140" s="3"/>
     </row>
-    <row r="141" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G141" s="3"/>
     </row>
-    <row r="142" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G142" s="3"/>
     </row>
-    <row r="143" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G143" s="3"/>
     </row>
-    <row r="144" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G144" s="3"/>
     </row>
-    <row r="145" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G145" s="3"/>
     </row>
-    <row r="146" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G146" s="3"/>
     </row>
-    <row r="147" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G147" s="3"/>
     </row>
-    <row r="148" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G148" s="3"/>
     </row>
-    <row r="154" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G154" s="3"/>
     </row>
-    <row r="160" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G160" s="3"/>
     </row>
-    <row r="162" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G162" s="3"/>
     </row>
-    <row r="163" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G163" s="3"/>
     </row>
-    <row r="165" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G165" s="3"/>
     </row>
-    <row r="173" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G173" s="3"/>
     </row>
-    <row r="174" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G174" s="3"/>
     </row>
-    <row r="177" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G177" s="3"/>
     </row>
-    <row r="178" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G178" s="3"/>
     </row>
-    <row r="181" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G181" s="3"/>
     </row>
-    <row r="182" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G182" s="3"/>
     </row>
-    <row r="186" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G186" s="3"/>
     </row>
-    <row r="188" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G188" s="3"/>
     </row>
-    <row r="193" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G193" s="3"/>
     </row>
-    <row r="196" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G196" s="3"/>
     </row>
-    <row r="200" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G200" s="3"/>
     </row>
-    <row r="202" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G202" s="3"/>
     </row>
-    <row r="203" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G203" s="3"/>
     </row>
-    <row r="207" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G207" s="3"/>
     </row>
-    <row r="208" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G208" s="3"/>
     </row>
-    <row r="209" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G209" s="3"/>
     </row>
-    <row r="210" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G210" s="3"/>
     </row>
-    <row r="211" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G211" s="3"/>
     </row>
-    <row r="212" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G212" s="3"/>
     </row>
-    <row r="213" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G213" s="3"/>
     </row>
-    <row r="214" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G214" s="3"/>
     </row>
-    <row r="217" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G217" s="3"/>
     </row>
-    <row r="219" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G219" s="3"/>
     </row>
-    <row r="223" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G223" s="3"/>
     </row>
-    <row r="224" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G224" s="3"/>
     </row>
-    <row r="227" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G227" s="3"/>
     </row>
-    <row r="228" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G228" s="3"/>
     </row>
-    <row r="229" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G229" s="3"/>
     </row>
-    <row r="231" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G231" s="3"/>
     </row>
-    <row r="232" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G232" s="3"/>
     </row>
-    <row r="234" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G234" s="3"/>
     </row>
-    <row r="237" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G237" s="3"/>
     </row>
-    <row r="238" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G238" s="3"/>
     </row>
-    <row r="239" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G239" s="3"/>
     </row>
-    <row r="240" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G240" s="3"/>
     </row>
-    <row r="242" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G242" s="3"/>
     </row>
-    <row r="243" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G243" s="3"/>
     </row>
-    <row r="244" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G244" s="3"/>
     </row>
-    <row r="247" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G247" s="3"/>
     </row>
-    <row r="248" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G248" s="3"/>
     </row>
-    <row r="249" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G249" s="3"/>
     </row>
-    <row r="251" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G251" s="3"/>
     </row>
-    <row r="252" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G252" s="3"/>
     </row>
-    <row r="253" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G253" s="3"/>
     </row>
-    <row r="254" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G254" s="3"/>
     </row>
-    <row r="255" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G255" s="3"/>
     </row>
-    <row r="256" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G256" s="3"/>
     </row>
-    <row r="260" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G260" s="3"/>
     </row>
-    <row r="261" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G261" s="3"/>
     </row>
-    <row r="262" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="262" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G262" s="3"/>
     </row>
-    <row r="266" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="266" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G266" s="3"/>
     </row>
-    <row r="267" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="267" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G267" s="3"/>
     </row>
-    <row r="268" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G268" s="3"/>
     </row>
-    <row r="282" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="282" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G282" s="3"/>
     </row>
-    <row r="283" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G283" s="3"/>
     </row>
-    <row r="284" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="284" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G284" s="3"/>
     </row>
-    <row r="285" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G285" s="3"/>
     </row>
-    <row r="286" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G286" s="3"/>
     </row>
-    <row r="287" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G287" s="3"/>
     </row>
-    <row r="289" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="289" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G289" s="3"/>
     </row>
-    <row r="292" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G292" s="3"/>
     </row>
-    <row r="293" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G293" s="3"/>
     </row>
-    <row r="294" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G294" s="3"/>
     </row>
-    <row r="295" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G295" s="3"/>
     </row>
-    <row r="297" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="297" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G297" s="3"/>
     </row>
-    <row r="298" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="298" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G298" s="3"/>
     </row>
-    <row r="299" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="299" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G299" s="3"/>
     </row>
-    <row r="300" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="300" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G300" s="3"/>
     </row>
-    <row r="301" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="301" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G301" s="3"/>
     </row>
-    <row r="302" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="302" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G302" s="3"/>
     </row>
-    <row r="303" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="303" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G303" s="3"/>
     </row>
-    <row r="305" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G305" s="3"/>
     </row>
-    <row r="306" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="306" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G306" s="3"/>
     </row>
-    <row r="307" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="307" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G307" s="3"/>
     </row>
-    <row r="308" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="308" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G308" s="3"/>
     </row>
-    <row r="309" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="309" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G309" s="3"/>
     </row>
-    <row r="310" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="310" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G310" s="3"/>
     </row>
-    <row r="311" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="311" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G311" s="3"/>
     </row>
-    <row r="312" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="312" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G312" s="3"/>
     </row>
-    <row r="313" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="313" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G313" s="3"/>
     </row>
-    <row r="314" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G314" s="3"/>
     </row>
-    <row r="315" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="315" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G315" s="3"/>
     </row>
-    <row r="316" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G316" s="3"/>
     </row>
-    <row r="317" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G317" s="3"/>
     </row>
-    <row r="318" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G318" s="3"/>
     </row>
-    <row r="319" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G319" s="3"/>
     </row>
-    <row r="320" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G320" s="3"/>
     </row>
-    <row r="321" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G321" s="3"/>
     </row>
-    <row r="323" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G323" s="3"/>
     </row>
-    <row r="324" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G324" s="3"/>
     </row>
-    <row r="326" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G326" s="3"/>
     </row>
-    <row r="327" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G327" s="3"/>
     </row>
-    <row r="330" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G330" s="3"/>
     </row>
-    <row r="331" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G331" s="3"/>
     </row>
-    <row r="332" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G332" s="3"/>
     </row>
-    <row r="333" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G333" s="3"/>
     </row>
-    <row r="334" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G334" s="3"/>
     </row>
-    <row r="335" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G335" s="3"/>
     </row>
-    <row r="336" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G336" s="3"/>
     </row>
-    <row r="337" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G337" s="3"/>
     </row>
-    <row r="338" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G338" s="3"/>
     </row>
-    <row r="346" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="346" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G346" s="3"/>
     </row>
-    <row r="370" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="370" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G370" s="3"/>
     </row>
-    <row r="371" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="371" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G371" s="3"/>
     </row>
-    <row r="372" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="372" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G372" s="3"/>
     </row>
-    <row r="373" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="373" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G373" s="3"/>
     </row>
-    <row r="374" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="374" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G374" s="3"/>
     </row>
-    <row r="375" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="375" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G375" s="3"/>
     </row>
-    <row r="376" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="376" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G376" s="3"/>
     </row>
-    <row r="377" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="377" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G377" s="3"/>
     </row>
-    <row r="378" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="378" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G378" s="3"/>
     </row>
-    <row r="379" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="379" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G379" s="3"/>
     </row>
-    <row r="380" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="380" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G380" s="3"/>
     </row>
-    <row r="381" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G381" s="3"/>
     </row>
-    <row r="382" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="382" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G382" s="3"/>
     </row>
-    <row r="383" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="383" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G383" s="3"/>
     </row>
-    <row r="384" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="384" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G384" s="3"/>
     </row>
-    <row r="385" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="385" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G385" s="3"/>
     </row>
-    <row r="386" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="386" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G386" s="3"/>
     </row>
-    <row r="387" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G387" s="3"/>
     </row>
-    <row r="388" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="388" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G388" s="3"/>
     </row>
-    <row r="389" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="389" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G389" s="3"/>
     </row>
-    <row r="390" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="390" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G390" s="3"/>
     </row>
-    <row r="391" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="391" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G391" s="3"/>
     </row>
-    <row r="392" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="392" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G392" s="3"/>
     </row>
-    <row r="393" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G393" s="3"/>
     </row>
-    <row r="394" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="394" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G394" s="3"/>
     </row>
-    <row r="395" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="395" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G395" s="3"/>
     </row>
-    <row r="396" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="396" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G396" s="3"/>
     </row>
-    <row r="397" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="397" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G397" s="3"/>
     </row>
-    <row r="398" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="398" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G398" s="3"/>
     </row>
-    <row r="399" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="399" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G399" s="3"/>
     </row>
-    <row r="400" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="400" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G400" s="3"/>
     </row>
-    <row r="401" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="401" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G401" s="3"/>
     </row>
-    <row r="402" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="402" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G402" s="3"/>
     </row>
-    <row r="404" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="404" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G404" s="3"/>
     </row>
-    <row r="405" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="405" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G405" s="3"/>
     </row>
-    <row r="406" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="406" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G406" s="3"/>
     </row>
-    <row r="407" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="407" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G407" s="3"/>
     </row>
-    <row r="408" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G408" s="3"/>
     </row>
-    <row r="409" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="409" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G409" s="3"/>
     </row>
-    <row r="410" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G410" s="3"/>
     </row>
-    <row r="411" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G411" s="3"/>
     </row>
-    <row r="412" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="412" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G412" s="3"/>
     </row>
-    <row r="413" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G413" s="3"/>
     </row>
-    <row r="414" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G414" s="3"/>
     </row>
-    <row r="415" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G415" s="3"/>
     </row>
-    <row r="417" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="417" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G417" s="3"/>
     </row>
-    <row r="418" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="418" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G418" s="3"/>
     </row>
-    <row r="419" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="419" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G419" s="3"/>
     </row>
-    <row r="420" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="420" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G420" s="3"/>
     </row>
-    <row r="421" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="421" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G421" s="3"/>
     </row>
-    <row r="422" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="422" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G422" s="3"/>
     </row>
-    <row r="423" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="423" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G423" s="3"/>
     </row>
-    <row r="424" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="424" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G424" s="3"/>
     </row>
-    <row r="425" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G425" s="3"/>
     </row>
-    <row r="426" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="426" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G426" s="3"/>
     </row>
-    <row r="427" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="427" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G427" s="3"/>
     </row>
-    <row r="428" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="428" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G428" s="3"/>
     </row>
-    <row r="429" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G429" s="3"/>
     </row>
-    <row r="430" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G430" s="3"/>
     </row>
-    <row r="431" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G431" s="3"/>
     </row>
-    <row r="432" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G432" s="3"/>
     </row>
-    <row r="434" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G434" s="3"/>
     </row>
-    <row r="435" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G435" s="3"/>
     </row>
-    <row r="436" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G436" s="3"/>
     </row>
-    <row r="437" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G437" s="3"/>
     </row>
-    <row r="438" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="438" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G438" s="3"/>
     </row>
-    <row r="439" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G439" s="3"/>
     </row>
-    <row r="440" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G440" s="3"/>
     </row>
-    <row r="441" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G441" s="3"/>
     </row>
-    <row r="442" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G442" s="3"/>
     </row>
-    <row r="443" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G443" s="3"/>
     </row>
-    <row r="444" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G444" s="3"/>
     </row>
-    <row r="445" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G445" s="3"/>
     </row>
-    <row r="446" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G446" s="3"/>
     </row>
-    <row r="447" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G447" s="3"/>
     </row>
-    <row r="448" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G448" s="3"/>
     </row>
-    <row r="449" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G449" s="3"/>
     </row>
-    <row r="450" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G450" s="3"/>
     </row>
-    <row r="451" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G451" s="3"/>
     </row>
-    <row r="452" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G452" s="3"/>
     </row>
-    <row r="453" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G453" s="3"/>
     </row>
-    <row r="454" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G454" s="3"/>
     </row>
-    <row r="455" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G455" s="3"/>
     </row>
-    <row r="456" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G456" s="3"/>
     </row>
-    <row r="457" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="457" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G457" s="3"/>
     </row>
-    <row r="458" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="458" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G458" s="3"/>
     </row>
-    <row r="459" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G459" s="3"/>
     </row>
-    <row r="460" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="460" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G460" s="3"/>
     </row>
-    <row r="461" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G461" s="3"/>
     </row>
-    <row r="462" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="462" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G462" s="3"/>
     </row>
-    <row r="463" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="463" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G463" s="3"/>
     </row>
-    <row r="464" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G464" s="3"/>
     </row>
-    <row r="466" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G466" s="3"/>
     </row>
-    <row r="467" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G467" s="3"/>
     </row>
-    <row r="468" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G468" s="3"/>
     </row>
-    <row r="469" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G469" s="3"/>
     </row>
-    <row r="470" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G470" s="3"/>
     </row>
-    <row r="471" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G471" s="3"/>
     </row>
-    <row r="472" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G472" s="3"/>
     </row>
-    <row r="473" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G473" s="3"/>
     </row>
-    <row r="474" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G474" s="3"/>
     </row>
-    <row r="475" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G475" s="3"/>
     </row>
-    <row r="476" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G476" s="3"/>
     </row>
-    <row r="477" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G477" s="3"/>
     </row>
-    <row r="478" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G478" s="3"/>
     </row>
-    <row r="479" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G479" s="3"/>
     </row>
-    <row r="480" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G480" s="3"/>
     </row>
-    <row r="481" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="481" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G481" s="3"/>
     </row>
-    <row r="482" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="482" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G482" s="3"/>
     </row>
-    <row r="483" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="483" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G483" s="3"/>
     </row>
-    <row r="484" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="484" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G484" s="3"/>
     </row>
-    <row r="485" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="485" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G485" s="3"/>
     </row>
-    <row r="486" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="486" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G486" s="3"/>
     </row>
-    <row r="487" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="487" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G487" s="3"/>
     </row>
-    <row r="489" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G489" s="3"/>
     </row>
-    <row r="490" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="490" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G490" s="3"/>
     </row>
-    <row r="491" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="491" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G491" s="3"/>
     </row>
-    <row r="492" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="492" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G492" s="3"/>
     </row>
-    <row r="493" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="493" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G493" s="3"/>
     </row>
-    <row r="494" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="494" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G494" s="3"/>
     </row>
-    <row r="495" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="495" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G495" s="3"/>
     </row>
-    <row r="496" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="496" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G496" s="3"/>
     </row>
-    <row r="497" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="497" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G497" s="3"/>
     </row>
-    <row r="498" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="498" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G498" s="3"/>
     </row>
-    <row r="499" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="499" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G499" s="3"/>
     </row>
-    <row r="500" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="500" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G500" s="3"/>
     </row>
-    <row r="501" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G501" s="3"/>
     </row>
-    <row r="502" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G502" s="3"/>
     </row>
-    <row r="504" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G504" s="3"/>
     </row>
-    <row r="505" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G505" s="3"/>
     </row>
-    <row r="506" ht="15" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G506" s="3"/>
     </row>
-    <row r="507" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="507" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F507" s="3"/>
       <c r="G507" s="3"/>
     </row>
-    <row r="508" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="508" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F508" s="3"/>
       <c r="G508" s="3"/>
     </row>
-    <row r="509" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="509" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F509" s="3"/>
       <c r="G509" s="3"/>
     </row>
-    <row r="510" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="510" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F510" s="3"/>
       <c r="G510" s="3"/>
     </row>
-    <row r="511" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="511" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F511" s="3"/>
       <c r="G511" s="3"/>
     </row>
-    <row r="512" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="512" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F512" s="3"/>
       <c r="G512" s="3"/>
     </row>
-    <row r="513" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="513" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F513" s="3"/>
       <c r="G513" s="3"/>
     </row>
-    <row r="514" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="514" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F514" s="3"/>
       <c r="G514" s="3"/>
     </row>
-    <row r="515" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="515" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F515" s="3"/>
       <c r="G515" s="3"/>
     </row>
-    <row r="516" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="516" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F516" s="3"/>
       <c r="G516" s="3"/>
     </row>
-    <row r="517" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="517" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F517" s="3"/>
       <c r="G517" s="3"/>
     </row>
-    <row r="518" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="518" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F518" s="3"/>
       <c r="G518" s="3"/>
     </row>
-    <row r="519" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="519" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F519" s="3"/>
       <c r="G519" s="3"/>
     </row>
-    <row r="520" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="520" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F520" s="3"/>
       <c r="G520" s="3"/>
     </row>
-    <row r="521" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="521" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F521" s="3"/>
       <c r="G521" s="3"/>
     </row>
-    <row r="522" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="522" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F522" s="3"/>
       <c r="G522" s="3"/>
     </row>
-    <row r="523" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="523" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F523" s="3"/>
       <c r="G523" s="3"/>
     </row>
-    <row r="524" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="524" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F524" s="3"/>
       <c r="G524" s="3"/>
     </row>
-    <row r="525" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="525" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F525" s="3"/>
       <c r="G525" s="3"/>
     </row>
-    <row r="526" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="526" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F526" s="3"/>
       <c r="G526" s="3"/>
     </row>
-    <row r="527" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="527" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F527" s="3"/>
       <c r="G527" s="3"/>
     </row>
-    <row r="528" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="528" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F528" s="3"/>
       <c r="G528" s="3"/>
     </row>
-    <row r="529" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="529" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F529" s="3"/>
       <c r="G529" s="3"/>
     </row>
-    <row r="530" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="530" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F530" s="3"/>
       <c r="G530" s="3"/>
     </row>
-    <row r="531" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="531" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F531" s="3"/>
       <c r="G531" s="3"/>
     </row>
-    <row r="532" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="532" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F532" s="3"/>
       <c r="G532" s="3"/>
     </row>
-    <row r="533" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="533" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F533" s="3"/>
       <c r="G533" s="3"/>
     </row>
-    <row r="534" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="534" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F534" s="3"/>
       <c r="G534" s="3"/>
     </row>
-    <row r="535" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="535" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F535" s="3"/>
       <c r="G535" s="3"/>
     </row>
-    <row r="536" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="536" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F536" s="3"/>
       <c r="G536" s="3"/>
     </row>
-    <row r="537" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="537" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F537" s="3"/>
       <c r="G537" s="3"/>
     </row>
-    <row r="538" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="538" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F538" s="3"/>
       <c r="G538" s="3"/>
     </row>
-    <row r="539" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="539" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F539" s="3"/>
       <c r="G539" s="3"/>
     </row>
-    <row r="540" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="540" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F540" s="3"/>
       <c r="G540" s="3"/>
     </row>
-    <row r="541" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="541" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F541" s="3"/>
       <c r="G541" s="3"/>
     </row>
-    <row r="542" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="542" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F542" s="3"/>
       <c r="G542" s="3"/>
     </row>
-    <row r="543" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="543" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F543" s="3"/>
       <c r="G543" s="3"/>
     </row>
-    <row r="544" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="544" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F544" s="3"/>
       <c r="G544" s="3"/>
     </row>
-    <row r="545" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="545" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F545" s="3"/>
       <c r="G545" s="3"/>
     </row>
-    <row r="546" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="546" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F546" s="3"/>
       <c r="G546" s="3"/>
     </row>
-    <row r="547" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="547" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F547" s="3"/>
       <c r="G547" s="3"/>
     </row>
-    <row r="548" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="548" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F548" s="3"/>
       <c r="G548" s="3"/>
     </row>
-    <row r="549" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="549" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F549" s="3"/>
       <c r="G549" s="3"/>
     </row>
-    <row r="550" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="550" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F550" s="3"/>
       <c r="G550" s="3"/>
     </row>
-    <row r="551" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="551" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F551" s="3"/>
       <c r="G551" s="3"/>
     </row>
-    <row r="552" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="552" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F552" s="3"/>
       <c r="G552" s="3"/>
     </row>
-    <row r="553" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="553" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F553" s="3"/>
       <c r="G553" s="3"/>
     </row>
-    <row r="554" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="554" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F554" s="3"/>
       <c r="G554" s="3"/>
     </row>
-    <row r="555" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="555" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F555" s="3"/>
       <c r="G555" s="3"/>
     </row>
-    <row r="556" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="556" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F556" s="3"/>
       <c r="G556" s="3"/>
     </row>
-    <row r="557" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="557" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F557" s="3"/>
       <c r="G557" s="3"/>
     </row>
-    <row r="558" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="558" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F558" s="3"/>
       <c r="G558" s="3"/>
     </row>
-    <row r="559" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="559" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F559" s="3"/>
       <c r="G559" s="3"/>
     </row>
-    <row r="560" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="560" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F560" s="3"/>
       <c r="G560" s="3"/>
     </row>
-    <row r="561" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="561" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F561" s="3"/>
       <c r="G561" s="3"/>
     </row>
-    <row r="562" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="562" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F562" s="3"/>
       <c r="G562" s="3"/>
     </row>
-    <row r="563" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="563" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F563" s="3"/>
       <c r="G563" s="3"/>
     </row>
-    <row r="564" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="564" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F564" s="3"/>
       <c r="G564" s="3"/>
     </row>
-    <row r="565" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="565" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F565" s="3"/>
       <c r="G565" s="3"/>
     </row>
-    <row r="566" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="566" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F566" s="3"/>
       <c r="G566" s="3"/>
     </row>
-    <row r="567" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="567" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F567" s="3"/>
       <c r="G567" s="3"/>
     </row>
-    <row r="568" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="568" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F568" s="3"/>
       <c r="G568" s="3"/>
     </row>
-    <row r="569" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="569" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F569" s="3"/>
       <c r="G569" s="3"/>
     </row>
-    <row r="570" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="570" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F570" s="3"/>
       <c r="G570" s="3"/>
     </row>
-    <row r="571" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="571" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F571" s="3"/>
       <c r="G571" s="3"/>
     </row>
-    <row r="572" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="572" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F572" s="3"/>
       <c r="G572" s="3"/>
     </row>
-    <row r="573" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="573" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F573" s="3"/>
       <c r="G573" s="3"/>
     </row>
-    <row r="574" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="574" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F574" s="3"/>
       <c r="G574" s="3"/>
     </row>
-    <row r="575" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="575" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F575" s="3"/>
       <c r="G575" s="3"/>
     </row>
-    <row r="576" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="576" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F576" s="3"/>
       <c r="G576" s="3"/>
     </row>
-    <row r="577" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="577" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F577" s="3"/>
       <c r="G577" s="3"/>
     </row>
-    <row r="578" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="578" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F578" s="3"/>
       <c r="G578" s="3"/>
     </row>
-    <row r="579" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="579" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F579" s="3"/>
       <c r="G579" s="3"/>
     </row>
-    <row r="580" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="580" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F580" s="3"/>
       <c r="G580" s="3"/>
     </row>
-    <row r="581" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="581" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F581" s="3"/>
       <c r="G581" s="3"/>
     </row>
-    <row r="582" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="582" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F582" s="3"/>
       <c r="G582" s="3"/>
     </row>
-    <row r="583" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="583" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F583" s="3"/>
       <c r="G583" s="3"/>
     </row>
-    <row r="584" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="584" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F584" s="3"/>
       <c r="G584" s="3"/>
     </row>
-    <row r="585" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="585" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F585" s="3"/>
       <c r="G585" s="3"/>
     </row>
-    <row r="586" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="586" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F586" s="3"/>
       <c r="G586" s="3"/>
     </row>
-    <row r="587" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="587" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F587" s="3"/>
       <c r="G587" s="3"/>
     </row>
-    <row r="588" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="588" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F588" s="3"/>
       <c r="G588" s="3"/>
     </row>
-    <row r="589" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="589" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F589" s="3"/>
       <c r="G589" s="3"/>
     </row>
-    <row r="590" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="590" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F590" s="3"/>
       <c r="G590" s="3"/>
     </row>
-    <row r="591" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="591" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F591" s="3"/>
       <c r="G591" s="3"/>
     </row>
-    <row r="592" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="592" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F592" s="3"/>
       <c r="G592" s="3"/>
     </row>
-    <row r="593" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="593" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F593" s="3"/>
       <c r="G593" s="3"/>
     </row>
-    <row r="594" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="594" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F594" s="3"/>
       <c r="G594" s="3"/>
     </row>
-    <row r="595" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="595" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F595" s="3"/>
       <c r="G595" s="3"/>
     </row>
-    <row r="596" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="596" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F596" s="3"/>
       <c r="G596" s="3"/>
     </row>
-    <row r="597" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="597" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F597" s="3"/>
       <c r="G597" s="3"/>
     </row>
-    <row r="598" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="598" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F598" s="3"/>
       <c r="G598" s="3"/>
     </row>
-    <row r="599" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="599" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F599" s="3"/>
       <c r="G599" s="3"/>
     </row>
-    <row r="600" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="600" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F600" s="3"/>
       <c r="G600" s="3"/>
     </row>
-    <row r="601" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="601" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F601" s="3"/>
       <c r="G601" s="3"/>
     </row>
-    <row r="602" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="602" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F602" s="3"/>
       <c r="G602" s="3"/>
     </row>
-    <row r="603" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="603" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F603" s="3"/>
       <c r="G603" s="3"/>
     </row>
-    <row r="604" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="604" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F604" s="3"/>
       <c r="G604" s="3"/>
     </row>
-    <row r="605" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="605" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F605" s="3"/>
       <c r="G605" s="3"/>
     </row>
-    <row r="606" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="606" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F606" s="3"/>
       <c r="G606" s="3"/>
     </row>
-    <row r="607" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="607" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F607" s="3"/>
       <c r="G607" s="3"/>
     </row>
-    <row r="608" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="608" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F608" s="3"/>
       <c r="G608" s="3"/>
     </row>
-    <row r="609" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="609" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F609" s="3"/>
       <c r="G609" s="3"/>
     </row>
-    <row r="610" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="610" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F610" s="3"/>
       <c r="G610" s="3"/>
     </row>
-    <row r="611" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="611" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F611" s="3"/>
       <c r="G611" s="3"/>
     </row>
-    <row r="612" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="612" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F612" s="3"/>
       <c r="G612" s="3"/>
     </row>
-    <row r="613" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="613" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F613" s="3"/>
       <c r="G613" s="3"/>
     </row>
-    <row r="614" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="614" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F614" s="3"/>
       <c r="G614" s="3"/>
     </row>
-    <row r="615" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="615" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F615" s="3"/>
       <c r="G615" s="3"/>
     </row>
-    <row r="616" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="616" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F616" s="3"/>
       <c r="G616" s="3"/>
     </row>
-    <row r="617" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="617" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F617" s="3"/>
       <c r="G617" s="3"/>
     </row>
-    <row r="618" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="618" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F618" s="3"/>
       <c r="G618" s="3"/>
     </row>
-    <row r="619" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="619" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F619" s="3"/>
       <c r="G619" s="3"/>
     </row>
-    <row r="620" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="620" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F620" s="3"/>
       <c r="G620" s="3"/>
     </row>
-    <row r="621" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="621" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F621" s="3"/>
       <c r="G621" s="3"/>
     </row>
-    <row r="622" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="622" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F622" s="3"/>
       <c r="G622" s="3"/>
     </row>
-    <row r="623" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="623" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F623" s="3"/>
       <c r="G623" s="3"/>
     </row>
-    <row r="624" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="624" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F624" s="3"/>
       <c r="G624" s="3"/>
     </row>
-    <row r="625" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="625" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F625" s="3"/>
       <c r="G625" s="3"/>
     </row>
-    <row r="626" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="626" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F626" s="3"/>
       <c r="G626" s="3"/>
     </row>
-    <row r="627" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="627" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F627" s="3"/>
       <c r="G627" s="3"/>
     </row>
-    <row r="628" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="628" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F628" s="3"/>
       <c r="G628" s="3"/>
     </row>
-    <row r="629" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="629" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F629" s="3"/>
       <c r="G629" s="3"/>
     </row>
-    <row r="630" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="630" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F630" s="3"/>
       <c r="G630" s="3"/>
     </row>
-    <row r="631" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="631" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F631" s="3"/>
       <c r="G631" s="3"/>
     </row>
-    <row r="632" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="632" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F632" s="3"/>
       <c r="G632" s="3"/>
     </row>
-    <row r="633" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="633" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F633" s="3"/>
       <c r="G633" s="3"/>
     </row>
-    <row r="634" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="634" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F634" s="3"/>
       <c r="G634" s="3"/>
     </row>
-    <row r="635" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="635" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F635" s="3"/>
       <c r="G635" s="3"/>
     </row>
-    <row r="636" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="636" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F636" s="3"/>
       <c r="G636" s="3"/>
     </row>
-    <row r="637" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="637" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F637" s="3"/>
       <c r="G637" s="3"/>
     </row>
-    <row r="638" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="638" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F638" s="3"/>
       <c r="G638" s="3"/>
     </row>
-    <row r="639" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="639" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F639" s="3"/>
       <c r="G639" s="3"/>
     </row>
-    <row r="640" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="640" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F640" s="3"/>
       <c r="G640" s="3"/>
     </row>
-    <row r="641" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="641" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F641" s="3"/>
       <c r="G641" s="3"/>
     </row>
-    <row r="642" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="642" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F642" s="3"/>
       <c r="G642" s="3"/>
     </row>
-    <row r="643" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="643" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F643" s="3"/>
       <c r="G643" s="3"/>
     </row>
-    <row r="644" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="644" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F644" s="3"/>
       <c r="G644" s="3"/>
     </row>
-    <row r="645" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="645" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F645" s="3"/>
       <c r="G645" s="3"/>
     </row>
-    <row r="646" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="646" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F646" s="3"/>
       <c r="G646" s="3"/>
     </row>
-    <row r="647" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="647" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F647" s="3"/>
       <c r="G647" s="3"/>
     </row>
-    <row r="648" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="648" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F648" s="3"/>
       <c r="G648" s="3"/>
     </row>
-    <row r="649" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="649" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F649" s="3"/>
       <c r="G649" s="3"/>
     </row>
-    <row r="650" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="650" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F650" s="3"/>
       <c r="G650" s="3"/>
     </row>
-    <row r="652" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="652" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F652" s="3"/>
       <c r="G652" s="3"/>
     </row>
-    <row r="653" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="653" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F653" s="3"/>
       <c r="G653" s="3"/>
     </row>
-    <row r="654" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="654" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F654" s="3"/>
       <c r="G654" s="3"/>
     </row>
-    <row r="655" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="655" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F655" s="3"/>
       <c r="G655" s="3"/>
     </row>
-    <row r="656" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="656" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F656" s="3"/>
       <c r="G656" s="3"/>
     </row>
-    <row r="657" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="657" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F657" s="3"/>
       <c r="G657" s="3"/>
     </row>
-    <row r="658" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="658" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F658" s="3"/>
       <c r="G658" s="3"/>
     </row>
-    <row r="659" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="659" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F659" s="3"/>
       <c r="G659" s="3"/>
     </row>
-    <row r="660" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="660" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F660" s="3"/>
       <c r="G660" s="3"/>
     </row>
-    <row r="661" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="661" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F661" s="3"/>
       <c r="G661" s="3"/>
     </row>
-    <row r="662" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="662" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F662" s="3"/>
       <c r="G662" s="3"/>
     </row>
-    <row r="663" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="663" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F663" s="3"/>
       <c r="G663" s="3"/>
     </row>
-    <row r="664" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="664" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F664" s="3"/>
       <c r="G664" s="3"/>
     </row>
-    <row r="665" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="665" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F665" s="3"/>
       <c r="G665" s="3"/>
     </row>
-    <row r="666" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="666" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F666" s="3"/>
       <c r="G666" s="3"/>
     </row>
-    <row r="667" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="667" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F667" s="3"/>
       <c r="G667" s="3"/>
     </row>
-    <row r="668" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="668" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F668" s="3"/>
       <c r="G668" s="3"/>
     </row>
-    <row r="669" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="669" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F669" s="3"/>
       <c r="G669" s="3"/>
     </row>
-    <row r="670" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="670" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F670" s="3"/>
       <c r="G670" s="3"/>
     </row>
-    <row r="671" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="671" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F671" s="3"/>
       <c r="G671" s="3"/>
     </row>
-    <row r="672" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="672" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F672" s="3"/>
       <c r="G672" s="3"/>
     </row>
-    <row r="673" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="673" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F673" s="3"/>
       <c r="G673" s="3"/>
     </row>
-    <row r="674" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="674" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F674" s="3"/>
       <c r="G674" s="3"/>
     </row>
-    <row r="675" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="675" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F675" s="3"/>
       <c r="G675" s="3"/>
     </row>
-    <row r="676" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="676" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F676" s="3"/>
       <c r="G676" s="3"/>
     </row>
-    <row r="677" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="677" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F677" s="3"/>
       <c r="G677" s="3"/>
     </row>
-    <row r="678" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="678" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F678" s="3"/>
       <c r="G678" s="3"/>
     </row>
-    <row r="679" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="679" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F679" s="3"/>
       <c r="G679" s="3"/>
     </row>
-    <row r="680" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="680" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F680" s="3"/>
       <c r="G680" s="3"/>
     </row>
-    <row r="681" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="681" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F681" s="3"/>
       <c r="G681" s="3"/>
     </row>
-    <row r="682" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="682" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F682" s="3"/>
       <c r="G682" s="3"/>
     </row>
-    <row r="683" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="683" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F683" s="3"/>
       <c r="G683" s="3"/>
     </row>
-    <row r="684" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="684" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F684" s="3"/>
       <c r="G684" s="3"/>
     </row>
-    <row r="685" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="685" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F685" s="3"/>
       <c r="G685" s="3"/>
     </row>
-    <row r="686" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="686" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F686" s="3"/>
       <c r="G686" s="3"/>
     </row>
-    <row r="687" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="687" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F687" s="3"/>
       <c r="G687" s="3"/>
     </row>
-    <row r="688" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="688" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F688" s="3"/>
       <c r="G688" s="3"/>
     </row>
-    <row r="689" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="689" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F689" s="3"/>
       <c r="G689" s="3"/>
     </row>
-    <row r="690" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="690" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F690" s="3"/>
       <c r="G690" s="3"/>
     </row>
-    <row r="691" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="691" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F691" s="3"/>
       <c r="G691" s="3"/>
     </row>
-    <row r="692" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="692" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F692" s="3"/>
       <c r="G692" s="3"/>
     </row>
-    <row r="693" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="693" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F693" s="3"/>
       <c r="G693" s="3"/>
     </row>
-    <row r="694" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="694" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F694" s="3"/>
       <c r="G694" s="3"/>
     </row>
-    <row r="695" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="695" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F695" s="3"/>
       <c r="G695" s="3"/>
     </row>
-    <row r="696" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="696" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F696" s="3"/>
       <c r="G696" s="3"/>
     </row>
-    <row r="697" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="697" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F697" s="3"/>
       <c r="G697" s="3"/>
     </row>
-    <row r="698" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="698" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F698" s="3"/>
       <c r="G698" s="3"/>
     </row>
-    <row r="699" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="699" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F699" s="3"/>
       <c r="G699" s="3"/>
     </row>
-    <row r="700" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="700" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F700" s="3"/>
       <c r="G700" s="3"/>
     </row>
-    <row r="701" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="701" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F701" s="3"/>
       <c r="G701" s="3"/>
     </row>
-    <row r="702" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="702" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F702" s="3"/>
       <c r="G702" s="3"/>
     </row>
-    <row r="703" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="703" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F703" s="3"/>
       <c r="G703" s="3"/>
     </row>
-    <row r="704" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="704" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F704" s="3"/>
       <c r="G704" s="3"/>
     </row>
-    <row r="705" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="705" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F705" s="3"/>
       <c r="G705" s="3"/>
     </row>
-    <row r="706" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="706" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F706" s="3"/>
       <c r="G706" s="3"/>
     </row>
-    <row r="707" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="707" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F707" s="3"/>
       <c r="G707" s="3"/>
     </row>
-    <row r="708" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="708" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F708" s="3"/>
       <c r="G708" s="3"/>
     </row>
-    <row r="709" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="709" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F709" s="3"/>
       <c r="G709" s="3"/>
     </row>
-    <row r="710" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="710" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F710" s="3"/>
       <c r="G710" s="3"/>
     </row>
-    <row r="711" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="711" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F711" s="3"/>
       <c r="G711" s="3"/>
     </row>
-    <row r="712" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="712" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F712" s="3"/>
       <c r="G712" s="3"/>
     </row>
-    <row r="713" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="713" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F713" s="3"/>
       <c r="G713" s="3"/>
     </row>
-    <row r="714" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="714" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F714" s="3"/>
       <c r="G714" s="3"/>
     </row>
-    <row r="715" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="715" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F715" s="3"/>
       <c r="G715" s="3"/>
     </row>
-    <row r="716" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="716" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F716" s="3"/>
       <c r="G716" s="3"/>
     </row>
-    <row r="717" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="717" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F717" s="3"/>
       <c r="G717" s="3"/>
     </row>
-    <row r="718" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="718" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F718" s="3"/>
       <c r="G718" s="3"/>
     </row>
-    <row r="719" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="719" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F719" s="3"/>
       <c r="G719" s="3"/>
     </row>
-    <row r="720" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="720" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F720" s="3"/>
       <c r="G720" s="3"/>
     </row>
-    <row r="721" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="721" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F721" s="3"/>
       <c r="G721" s="3"/>
     </row>
-    <row r="722" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="722" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F722" s="3"/>
       <c r="G722" s="3"/>
     </row>
-    <row r="723" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="723" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F723" s="3"/>
       <c r="G723" s="3"/>
     </row>
-    <row r="724" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="724" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F724" s="3"/>
       <c r="G724" s="3"/>
     </row>
-    <row r="725" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="725" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F725" s="3"/>
       <c r="G725" s="3"/>
     </row>
-    <row r="726" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="726" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F726" s="3"/>
       <c r="G726" s="3"/>
     </row>
-    <row r="727" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="727" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F727" s="3"/>
       <c r="G727" s="3"/>
     </row>
-    <row r="728" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="728" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F728" s="3"/>
       <c r="G728" s="3"/>
     </row>
-    <row r="729" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="729" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F729" s="3"/>
       <c r="G729" s="3"/>
     </row>
-    <row r="730" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="730" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F730" s="3"/>
       <c r="G730" s="3"/>
     </row>
-    <row r="731" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="731" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F731" s="3"/>
       <c r="G731" s="3"/>
     </row>
-    <row r="732" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="732" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F732" s="3"/>
       <c r="G732" s="3"/>
     </row>
-    <row r="733" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="733" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F733" s="3"/>
       <c r="G733" s="3"/>
     </row>
-    <row r="734" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="734" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F734" s="3"/>
       <c r="G734" s="3"/>
     </row>
-    <row r="735" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="735" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F735" s="3"/>
       <c r="G735" s="3"/>
     </row>
-    <row r="736" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="736" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F736" s="3"/>
       <c r="G736" s="3"/>
     </row>
-    <row r="737" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="737" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F737" s="3"/>
       <c r="G737" s="3"/>
     </row>
-    <row r="738" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="738" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F738" s="3"/>
       <c r="G738" s="3"/>
     </row>
-    <row r="739" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="739" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F739" s="3"/>
       <c r="G739" s="3"/>
     </row>
-    <row r="740" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="740" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F740" s="3"/>
       <c r="G740" s="3"/>
     </row>
-    <row r="741" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="741" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F741" s="3"/>
       <c r="G741" s="3"/>
     </row>
-    <row r="742" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="742" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F742" s="3"/>
       <c r="G742" s="3"/>
     </row>
-    <row r="743" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="743" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F743" s="3"/>
       <c r="G743" s="3"/>
     </row>
-    <row r="744" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="744" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F744" s="3"/>
       <c r="G744" s="3"/>
     </row>
-    <row r="745" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="745" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F745" s="3"/>
       <c r="G745" s="3"/>
     </row>
-    <row r="746" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="746" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F746" s="3"/>
       <c r="G746" s="3"/>
     </row>
-    <row r="747" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="747" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F747" s="3"/>
       <c r="G747" s="3"/>
     </row>
-    <row r="748" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="748" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F748" s="3"/>
       <c r="G748" s="3"/>
     </row>
-    <row r="749" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="749" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F749" s="3"/>
       <c r="G749" s="3"/>
     </row>
-    <row r="750" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="750" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F750" s="3"/>
       <c r="G750" s="3"/>
     </row>
-    <row r="751" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="751" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F751" s="3"/>
       <c r="G751" s="3"/>
     </row>
-    <row r="752" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="752" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F752" s="3"/>
       <c r="G752" s="3"/>
     </row>
-    <row r="753" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="753" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F753" s="3"/>
       <c r="G753" s="3"/>
     </row>
-    <row r="754" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="754" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F754" s="3"/>
       <c r="G754" s="3"/>
     </row>
-    <row r="755" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="755" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F755" s="3"/>
       <c r="G755" s="3"/>
     </row>
-    <row r="756" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="756" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F756" s="3"/>
       <c r="G756" s="3"/>
     </row>
-    <row r="757" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="757" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F757" s="3"/>
       <c r="G757" s="3"/>
     </row>
-    <row r="758" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="758" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F758" s="3"/>
       <c r="G758" s="3"/>
     </row>
-    <row r="759" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="759" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F759" s="3"/>
       <c r="G759" s="3"/>
     </row>
-    <row r="760" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="760" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F760" s="3"/>
       <c r="G760" s="3"/>
     </row>
-    <row r="761" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="761" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F761" s="3"/>
       <c r="G761" s="3"/>
     </row>
-    <row r="762" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="762" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F762" s="3"/>
       <c r="G762" s="3"/>
     </row>
-    <row r="763" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="763" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F763" s="3"/>
       <c r="G763" s="3"/>
     </row>
-    <row r="764" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="764" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F764" s="3"/>
       <c r="G764" s="3"/>
     </row>
-    <row r="765" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="765" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F765" s="3"/>
       <c r="G765" s="3"/>
     </row>
-    <row r="766" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="766" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F766" s="3"/>
       <c r="G766" s="3"/>
     </row>
-    <row r="767" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="767" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F767" s="3"/>
       <c r="G767" s="3"/>
     </row>
-    <row r="768" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="768" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F768" s="3"/>
       <c r="G768" s="3"/>
     </row>
-    <row r="769" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="769" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F769" s="3"/>
       <c r="G769" s="3"/>
     </row>
-    <row r="770" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="770" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F770" s="3"/>
       <c r="G770" s="3"/>
     </row>
-    <row r="771" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="771" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F771" s="3"/>
       <c r="G771" s="3"/>
     </row>
-    <row r="772" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="772" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F772" s="3"/>
       <c r="G772" s="3"/>
     </row>
-    <row r="773" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="773" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F773" s="3"/>
       <c r="G773" s="3"/>
     </row>
-    <row r="774" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="774" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F774" s="3"/>
       <c r="G774" s="3"/>
     </row>
-    <row r="775" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="775" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F775" s="3"/>
       <c r="G775" s="3"/>
     </row>
-    <row r="776" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="776" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F776" s="3"/>
       <c r="G776" s="3"/>
     </row>
-    <row r="777" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="777" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F777" s="3"/>
       <c r="G777" s="3"/>
     </row>
-    <row r="778" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="778" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F778" s="3"/>
       <c r="G778" s="3"/>
     </row>
-    <row r="779" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="779" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F779" s="3"/>
       <c r="G779" s="3"/>
     </row>
-    <row r="780" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="780" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F780" s="3"/>
       <c r="G780" s="3"/>
     </row>
-    <row r="781" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="781" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F781" s="3"/>
       <c r="G781" s="3"/>
     </row>
-    <row r="782" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="782" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F782" s="3"/>
       <c r="G782" s="3"/>
     </row>
-    <row r="812" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="812" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F812" s="3"/>
       <c r="G812" s="3"/>
     </row>
-    <row r="818" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="818" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F818" s="3"/>
       <c r="G818" s="3"/>
     </row>
-    <row r="819" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="819" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F819" s="3"/>
       <c r="G819" s="3"/>
     </row>
-    <row r="823" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="823" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F823" s="3"/>
       <c r="G823" s="3"/>
     </row>
-    <row r="824" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="824" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F824" s="3"/>
       <c r="G824" s="3"/>
     </row>
-    <row r="845" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="845" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F845" s="3"/>
       <c r="G845" s="3"/>
     </row>
-    <row r="849" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="849" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F849" s="3"/>
       <c r="G849" s="3"/>
     </row>
-    <row r="855" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="855" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F855" s="3"/>
       <c r="G855" s="3"/>
     </row>
-    <row r="859" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="859" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F859" s="3"/>
       <c r="G859" s="3"/>
     </row>
-    <row r="860" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="860" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F860" s="3"/>
       <c r="G860" s="3"/>
     </row>
-    <row r="863" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="863" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F863" s="3"/>
       <c r="G863" s="3"/>
     </row>
-    <row r="864" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="864" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F864" s="3"/>
       <c r="G864" s="3"/>
     </row>
-    <row r="869" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="869" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F869" s="3"/>
       <c r="G869" s="3"/>
     </row>
-    <row r="871" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="871" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F871" s="3"/>
       <c r="G871" s="3"/>
     </row>
-    <row r="879" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="879" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F879" s="3"/>
       <c r="G879" s="3"/>
     </row>
-    <row r="880" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="880" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F880" s="3"/>
       <c r="G880" s="3"/>
     </row>
-    <row r="881" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="881" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F881" s="3"/>
       <c r="G881" s="3"/>
     </row>
-    <row r="882" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="882" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F882" s="3"/>
       <c r="G882" s="3"/>
     </row>
-    <row r="883" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="883" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F883" s="3"/>
       <c r="G883" s="3"/>
     </row>
-    <row r="884" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="884" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F884" s="3"/>
       <c r="G884" s="3"/>
     </row>
-    <row r="885" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="885" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F885" s="3"/>
       <c r="G885" s="3"/>
     </row>
-    <row r="886" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="886" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F886" s="3"/>
       <c r="G886" s="3"/>
     </row>
-    <row r="887" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="887" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F887" s="3"/>
       <c r="G887" s="3"/>
     </row>
-    <row r="888" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="888" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F888" s="3"/>
       <c r="G888" s="3"/>
     </row>
-    <row r="889" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="889" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F889" s="3"/>
       <c r="G889" s="3"/>
     </row>
-    <row r="890" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="890" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F890" s="3"/>
       <c r="G890" s="3"/>
     </row>
-    <row r="891" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="891" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F891" s="3"/>
       <c r="G891" s="3"/>
     </row>
-    <row r="892" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="892" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F892" s="3"/>
       <c r="G892" s="3"/>
     </row>
-    <row r="893" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="893" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F893" s="3"/>
       <c r="G893" s="3"/>
     </row>
-    <row r="894" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="894" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F894" s="3"/>
       <c r="G894" s="3"/>
     </row>
-    <row r="895" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="895" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F895" s="3"/>
       <c r="G895" s="3"/>
     </row>
-    <row r="896" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="896" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F896" s="3"/>
       <c r="G896" s="3"/>
     </row>
-    <row r="897" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="897" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F897" s="3"/>
       <c r="G897" s="3"/>
     </row>
-    <row r="898" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="898" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F898" s="3"/>
       <c r="G898" s="3"/>
     </row>
-    <row r="899" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="899" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F899" s="3"/>
       <c r="G899" s="3"/>
     </row>
-    <row r="900" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="900" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F900" s="3"/>
       <c r="G900" s="3"/>
     </row>
-    <row r="901" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="901" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F901" s="3"/>
       <c r="G901" s="3"/>
     </row>
-    <row r="902" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="902" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F902" s="3"/>
       <c r="G902" s="3"/>
     </row>
-    <row r="903" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="903" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F903" s="3"/>
       <c r="G903" s="3"/>
     </row>
-    <row r="904" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="904" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F904" s="3"/>
       <c r="G904" s="3"/>
     </row>
-    <row r="905" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="905" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F905" s="3"/>
       <c r="G905" s="3"/>
     </row>
-    <row r="906" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="906" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F906" s="3"/>
       <c r="G906" s="3"/>
     </row>
-    <row r="907" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="907" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F907" s="3"/>
       <c r="G907" s="3"/>
     </row>
-    <row r="908" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="908" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F908" s="3"/>
       <c r="G908" s="3"/>
     </row>
-    <row r="909" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="909" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F909" s="3"/>
       <c r="G909" s="3"/>
     </row>
-    <row r="910" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="910" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F910" s="3"/>
       <c r="G910" s="3"/>
     </row>
-    <row r="911" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="911" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F911" s="3"/>
       <c r="G911" s="3"/>
     </row>
-    <row r="912" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="912" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F912" s="3"/>
       <c r="G912" s="3"/>
     </row>
-    <row r="913" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="913" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F913" s="3"/>
       <c r="G913" s="3"/>
     </row>
-    <row r="914" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="914" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F914" s="3"/>
       <c r="G914" s="3"/>
     </row>
-    <row r="915" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="915" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F915" s="3"/>
       <c r="G915" s="3"/>
     </row>
-    <row r="916" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="916" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F916" s="3"/>
       <c r="G916" s="3"/>
     </row>
-    <row r="917" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="917" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F917" s="3"/>
       <c r="G917" s="3"/>
     </row>
-    <row r="918" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="918" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F918" s="3"/>
       <c r="G918" s="3"/>
     </row>
-    <row r="919" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="919" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F919" s="3"/>
       <c r="G919" s="3"/>
     </row>
-    <row r="920" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="920" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F920" s="3"/>
       <c r="G920" s="3"/>
     </row>
-    <row r="921" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="921" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F921" s="3"/>
       <c r="G921" s="3"/>
     </row>
-    <row r="922" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="922" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F922" s="3"/>
       <c r="G922" s="3"/>
     </row>
-    <row r="923" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="923" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F923" s="3"/>
       <c r="G923" s="3"/>
     </row>
-    <row r="924" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="924" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F924" s="3"/>
       <c r="G924" s="3"/>
     </row>
-    <row r="925" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="925" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F925" s="3"/>
       <c r="G925" s="3"/>
     </row>
-    <row r="926" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="926" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F926" s="3"/>
       <c r="G926" s="3"/>
     </row>
-    <row r="927" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="927" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F927" s="3"/>
       <c r="G927" s="3"/>
     </row>
-    <row r="928" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="928" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F928" s="3"/>
       <c r="G928" s="3"/>
     </row>
-    <row r="929" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="929" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F929" s="3"/>
       <c r="G929" s="3"/>
     </row>
-    <row r="930" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="930" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F930" s="3"/>
       <c r="G930" s="3"/>
     </row>
-    <row r="931" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="931" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F931" s="3"/>
       <c r="G931" s="3"/>
     </row>
-    <row r="932" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="932" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F932" s="3"/>
       <c r="G932" s="3"/>
     </row>
-    <row r="933" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="933" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F933" s="3"/>
       <c r="G933" s="3"/>
     </row>
-    <row r="934" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="934" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F934" s="3"/>
       <c r="G934" s="3"/>
     </row>
-    <row r="935" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="935" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F935" s="3"/>
       <c r="G935" s="3"/>
     </row>
-    <row r="936" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="936" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F936" s="3"/>
       <c r="G936" s="3"/>
     </row>
-    <row r="937" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="937" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F937" s="3"/>
       <c r="G937" s="3"/>
     </row>
-    <row r="938" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="938" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F938" s="3"/>
       <c r="G938" s="3"/>
     </row>
-    <row r="939" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="939" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F939" s="3"/>
       <c r="G939" s="3"/>
     </row>
-    <row r="940" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="940" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F940" s="3"/>
       <c r="G940" s="3"/>
     </row>
-    <row r="941" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="941" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F941" s="3"/>
       <c r="G941" s="3"/>
     </row>
-    <row r="942" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="942" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F942" s="3"/>
       <c r="G942" s="3"/>
     </row>
-    <row r="943" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="943" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F943" s="3"/>
       <c r="G943" s="3"/>
     </row>
-    <row r="944" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="944" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F944" s="3"/>
       <c r="G944" s="3"/>
     </row>
-    <row r="945" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="945" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F945" s="3"/>
       <c r="G945" s="3"/>
     </row>
-    <row r="946" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="946" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F946" s="3"/>
       <c r="G946" s="3"/>
     </row>
-    <row r="947" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="947" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F947" s="3"/>
       <c r="G947" s="3"/>
     </row>
-    <row r="948" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="948" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F948" s="3"/>
       <c r="G948" s="3"/>
     </row>
-    <row r="949" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="949" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F949" s="3"/>
       <c r="G949" s="3"/>
     </row>
-    <row r="950" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="950" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F950" s="3"/>
       <c r="G950" s="3"/>
     </row>
-    <row r="951" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="951" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F951" s="3"/>
       <c r="G951" s="3"/>
     </row>
-    <row r="952" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="952" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F952" s="3"/>
       <c r="G952" s="3"/>
     </row>
-    <row r="953" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="953" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F953" s="3"/>
       <c r="G953" s="3"/>
     </row>
-    <row r="954" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="954" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F954" s="3"/>
       <c r="G954" s="3"/>
     </row>
-    <row r="955" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="955" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F955" s="3"/>
       <c r="G955" s="3"/>
     </row>
-    <row r="956" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="956" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F956" s="3"/>
       <c r="G956" s="3"/>
     </row>
-    <row r="957" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="957" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F957" s="3"/>
       <c r="G957" s="3"/>
     </row>
-    <row r="958" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="958" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F958" s="3"/>
       <c r="G958" s="3"/>
     </row>
-    <row r="959" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="959" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F959" s="3"/>
       <c r="G959" s="3"/>
     </row>
-    <row r="960" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="960" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F960" s="3"/>
       <c r="G960" s="3"/>
     </row>
-    <row r="961" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="961" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F961" s="3"/>
       <c r="G961" s="3"/>
     </row>
-    <row r="962" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="962" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F962" s="3"/>
       <c r="G962" s="3"/>
     </row>
-    <row r="963" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="963" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F963" s="3"/>
       <c r="G963" s="3"/>
     </row>
-    <row r="964" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="964" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F964" s="3"/>
       <c r="G964" s="3"/>
     </row>
-    <row r="965" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="965" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F965" s="3"/>
       <c r="G965" s="3"/>
     </row>
-    <row r="966" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="966" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F966" s="3"/>
       <c r="G966" s="3"/>
     </row>
-    <row r="967" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="967" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F967" s="3"/>
       <c r="G967" s="3"/>
     </row>
-    <row r="968" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="968" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F968" s="3"/>
       <c r="G968" s="3"/>
     </row>
-    <row r="969" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="969" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F969" s="3"/>
       <c r="G969" s="3"/>
     </row>
-    <row r="970" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="970" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F970" s="3"/>
       <c r="G970" s="3"/>
     </row>
-    <row r="971" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="971" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F971" s="3"/>
       <c r="G971" s="3"/>
     </row>
-    <row r="972" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="972" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F972" s="3"/>
       <c r="G972" s="3"/>
     </row>
-    <row r="973" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="973" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F973" s="3"/>
       <c r="G973" s="3"/>
     </row>
-    <row r="974" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="974" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F974" s="3"/>
       <c r="G974" s="3"/>
     </row>
-    <row r="975" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="975" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F975" s="3"/>
       <c r="G975" s="3"/>
     </row>
-    <row r="976" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="976" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F976" s="3"/>
       <c r="G976" s="3"/>
     </row>
-    <row r="977" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="977" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F977" s="3"/>
       <c r="G977" s="3"/>
     </row>
-    <row r="978" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="978" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F978" s="3"/>
       <c r="G978" s="3"/>
     </row>
-    <row r="979" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="979" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F979" s="3"/>
       <c r="G979" s="3"/>
     </row>
-    <row r="980" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="980" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F980" s="3"/>
       <c r="G980" s="3"/>
     </row>
-    <row r="981" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="981" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F981" s="3"/>
       <c r="G981" s="3"/>
     </row>
-    <row r="982" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="982" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F982" s="3"/>
       <c r="G982" s="3"/>
     </row>
-    <row r="983" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="983" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F983" s="3"/>
       <c r="G983" s="3"/>
     </row>
-    <row r="984" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="984" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F984" s="3"/>
       <c r="G984" s="3"/>
     </row>
-    <row r="985" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="985" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F985" s="3"/>
       <c r="G985" s="3"/>
     </row>
-    <row r="986" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="986" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F986" s="3"/>
       <c r="G986" s="3"/>
     </row>
-    <row r="987" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="987" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F987" s="3"/>
       <c r="G987" s="3"/>
     </row>
-    <row r="988" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="988" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F988" s="3"/>
       <c r="G988" s="3"/>
     </row>
-    <row r="989" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="989" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F989" s="3"/>
       <c r="G989" s="3"/>
     </row>
-    <row r="990" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="990" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F990" s="3"/>
       <c r="G990" s="3"/>
     </row>
-    <row r="991" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="991" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F991" s="3"/>
       <c r="G991" s="3"/>
     </row>
-    <row r="992" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="992" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F992" s="3"/>
       <c r="G992" s="3"/>
     </row>
-    <row r="993" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="993" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F993" s="3"/>
       <c r="G993" s="3"/>
     </row>
-    <row r="994" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="994" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F994" s="3"/>
       <c r="G994" s="3"/>
     </row>
-    <row r="995" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="995" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F995" s="3"/>
       <c r="G995" s="3"/>
     </row>
-    <row r="996" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="996" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F996" s="3"/>
       <c r="G996" s="3"/>
     </row>
-    <row r="997" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="997" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F997" s="3"/>
       <c r="G997" s="3"/>
     </row>
-    <row r="998" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="998" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F998" s="3"/>
       <c r="G998" s="3"/>
     </row>
-    <row r="999" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="999" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F999" s="3"/>
       <c r="G999" s="3"/>
     </row>
-    <row r="1000" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="1000" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F1000" s="3"/>
       <c r="G1000" s="3"/>
     </row>
-    <row r="1001" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="1001" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F1001" s="3"/>
       <c r="G1001" s="3"/>
     </row>
-    <row r="1002" ht="15" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="1002" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F1002" s="3"/>
       <c r="G1002" s="3"/>
     </row>
-    <row r="1048576" ht="12.8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>